<commit_message>
Fixing Presence sheet with signature
</commit_message>
<xml_diff>
--- a/backend/src/templates/feuille_presence_template.xlsx
+++ b/backend/src/templates/feuille_presence_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\excellia-app\backend\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A804BC4-33D7-4BA5-A580-2AF9241F4E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333B49C9-1D04-4614-B336-04F96F16DDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="50">
   <si>
     <t>Feuille de présence mission</t>
   </si>
@@ -34,6 +34,9 @@
     <t>Référence engagement (BC/Contrat/ Convention)</t>
   </si>
   <si>
+    <t>2025/11/0060</t>
+  </si>
+  <si>
     <t>Département ou service</t>
   </si>
   <si>
@@ -43,13 +46,13 @@
     <t>Responsable suivi de mission (Banque Zitouna)</t>
   </si>
   <si>
-    <t>Mohamed Salah Mhamedi</t>
+    <t>Moez Dhehibi</t>
   </si>
   <si>
     <t>Période objet de la facturation</t>
   </si>
   <si>
-    <t>Décember-2025</t>
+    <t>Février 2026</t>
   </si>
   <si>
     <t>Date</t>
@@ -58,7 +61,13 @@
     <t>Tâches et livrables</t>
   </si>
   <si>
-    <t>01 du mois</t>
+    <t>Temps</t>
+  </si>
+  <si>
+    <t>01 du mois (Dimanche)</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>02 du mois</t>
@@ -73,7 +82,13 @@
     <t>05 du mois</t>
   </si>
   <si>
-    <t>08 du mois</t>
+    <t>06 du mois</t>
+  </si>
+  <si>
+    <t>07 du mois (Samedi)</t>
+  </si>
+  <si>
+    <t>08 du mois (Dimanche)</t>
   </si>
   <si>
     <t>09 du mois</t>
@@ -88,7 +103,13 @@
     <t>12 du mois</t>
   </si>
   <si>
-    <t>15 du mois</t>
+    <t>13 du mois</t>
+  </si>
+  <si>
+    <t>14 du mois (Samedi)</t>
+  </si>
+  <si>
+    <t>15 du mois (Dimanche)</t>
   </si>
   <si>
     <t>16 du mois</t>
@@ -103,7 +124,13 @@
     <t>19 du mois</t>
   </si>
   <si>
-    <t>22 du mois</t>
+    <t>20 du mois</t>
+  </si>
+  <si>
+    <t>21 du mois (Samedi)</t>
+  </si>
+  <si>
+    <t>22 du mois (Dimanche)</t>
   </si>
   <si>
     <t>23 du mois</t>
@@ -118,52 +145,31 @@
     <t>26 du mois</t>
   </si>
   <si>
-    <t>29 du mois</t>
-  </si>
-  <si>
-    <t>30 du mois</t>
-  </si>
-  <si>
-    <t>31 du mois</t>
+    <t>27 du mois</t>
+  </si>
+  <si>
+    <t>28 du mois (Samedi)</t>
+  </si>
+  <si>
+    <t>Congé</t>
+  </si>
+  <si>
+    <t>Total jours travaillés</t>
+  </si>
+  <si>
+    <t>Responsable d'équipe</t>
   </si>
   <si>
     <t>Responsable suivi de mission</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
+    <t>Aymen Selmi</t>
   </si>
   <si>
     <t>Date de signature</t>
   </si>
   <si>
     <t>Signature</t>
-  </si>
-  <si>
-    <t>Temps</t>
-  </si>
-  <si>
-    <t>28 du mois</t>
-  </si>
-  <si>
-    <t>27 du mois</t>
-  </si>
-  <si>
-    <t>06 du mois</t>
-  </si>
-  <si>
-    <t>07 du mois</t>
-  </si>
-  <si>
-    <t>13 du mois</t>
-  </si>
-  <si>
-    <t>14 du mois</t>
-  </si>
-  <si>
-    <t>20 du mois</t>
-  </si>
-  <si>
-    <t>21 du mois</t>
   </si>
 </sst>
 </file>
@@ -173,7 +179,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -226,18 +232,13 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial Narrow"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial Narrow"/>
     </font>
@@ -285,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -425,7 +426,9 @@
       <top style="hair">
         <color rgb="FF9BBB59"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -434,7 +437,9 @@
       <top style="hair">
         <color rgb="FF9BBB59"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -457,6 +462,26 @@
         <color rgb="FF9BBB59"/>
       </left>
       <right/>
+      <top style="hair">
+        <color rgb="FF9BBB59"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="FF9BBB59"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF9BBB59"/>
+      </left>
+      <right/>
       <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
@@ -473,41 +498,37 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color rgb="FF9BBB59"/>
-      </left>
+      <left/>
       <right/>
-      <top style="hair">
-        <color rgb="FF9BBB59"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FF9BBB59"/>
+      </left>
       <right/>
-      <top style="hair">
+      <top style="thin">
         <color rgb="FF9BBB59"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF9BBB59"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF9BBB59"/>
       </left>
-      <right style="hair">
+      <right style="thin">
         <color rgb="FF9BBB59"/>
       </right>
-      <top style="hair">
+      <top style="thin">
         <color rgb="FF9BBB59"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF9BBB59"/>
       </bottom>
       <diagonal/>
     </border>
@@ -518,10 +539,10 @@
       <right style="thin">
         <color rgb="FF9BBB59"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF9BBB59"/>
-      </bottom>
+      <top style="thin">
+        <color rgb="FF9BBB59"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -531,25 +552,10 @@
       <right style="thin">
         <color rgb="FF9BBB59"/>
       </right>
-      <top style="thin">
-        <color rgb="FF9BBB59"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color rgb="FF9BBB59"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF9BBB59"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF9BBB59"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF9BBB59"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -567,7 +573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -590,8 +596,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -599,20 +605,20 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -636,27 +642,33 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -673,6 +685,53 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2743200" cy="1318260"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="image1.png" title="Image">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2293620" y="14813280"/>
+          <a:ext cx="2743200" cy="1318260"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -876,7 +935,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D1000"/>
+  <dimension ref="A1:D997"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -885,7 +944,7 @@
     <col min="5" max="6" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.4">
+    <row r="1" spans="1:4" ht="14.25" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
     </row>
@@ -897,11 +956,12 @@
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
     </row>
-    <row r="4" spans="1:4" ht="14.4">
+    <row r="3" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:4" ht="14.25" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="15.6">
+    <row r="5" spans="1:4" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -910,556 +970,652 @@
       </c>
       <c r="C5" s="19"/>
     </row>
-    <row r="6" spans="1:4" ht="14.4">
+    <row r="6" spans="1:4" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20"/>
+      <c r="B6" s="20" t="s">
+        <v>4</v>
+      </c>
       <c r="C6" s="19"/>
     </row>
-    <row r="7" spans="1:4" ht="14.4">
+    <row r="7" spans="1:4" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="19"/>
     </row>
-    <row r="8" spans="1:4" ht="14.4">
+    <row r="8" spans="1:4" ht="14.25" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="1:4" ht="14.4">
+    <row r="9" spans="1:4" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="19"/>
     </row>
-    <row r="10" spans="1:4" ht="14.4">
+    <row r="10" spans="1:4" ht="14.25" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="1:4" ht="14.4">
+    <row r="11" spans="1:4" ht="14.25" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
     </row>
     <row r="12" spans="1:4" ht="20.25" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="24"/>
       <c r="D12" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30" customHeight="1">
+      <c r="A13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="26"/>
+      <c r="D13" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="30" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="26"/>
+      <c r="D14" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="30" customHeight="1">
+      <c r="A15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="26"/>
+      <c r="D15" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="30" customHeight="1">
+      <c r="A16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="26"/>
+      <c r="D16" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="30" customHeight="1">
+      <c r="A17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="26"/>
+      <c r="D17" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="30" customHeight="1">
+      <c r="A18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="26"/>
+      <c r="D18" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="30" customHeight="1">
+      <c r="A19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="26"/>
+      <c r="D19" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="30" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="26"/>
+      <c r="D20" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="30" customHeight="1">
+      <c r="A21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="26"/>
+      <c r="D21" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="30" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="26"/>
+      <c r="D22" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="30" customHeight="1">
+      <c r="A23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="26"/>
+      <c r="D23" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="30" customHeight="1">
+      <c r="A24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="26"/>
+      <c r="D24" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="30" customHeight="1">
+      <c r="A25" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="26"/>
+      <c r="D25" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="30" customHeight="1">
+      <c r="A26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="26"/>
+      <c r="D26" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="30" customHeight="1">
+      <c r="A27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="29"/>
+      <c r="D27" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="30" customHeight="1">
+      <c r="A28" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="30"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="8"/>
+    </row>
+    <row r="29" spans="1:4" ht="30" customHeight="1">
+      <c r="A29" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="8"/>
+    </row>
+    <row r="30" spans="1:4" ht="30" customHeight="1">
+      <c r="A30" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="30"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="8"/>
+    </row>
+    <row r="31" spans="1:4" ht="30" customHeight="1">
+      <c r="A31" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="30"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="8"/>
+    </row>
+    <row r="32" spans="1:4" ht="30" customHeight="1">
+      <c r="A32" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="30"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="8"/>
+    </row>
+    <row r="33" spans="1:4" ht="30" customHeight="1">
+      <c r="A33" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="30"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="30" customHeight="1">
+      <c r="A34" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="31"/>
+      <c r="D34" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="30" customHeight="1">
+      <c r="A35" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="26"/>
+      <c r="D35" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="30" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="26"/>
+      <c r="D36" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="30" customHeight="1">
+      <c r="A37" s="6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="18" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="7"/>
-    </row>
-    <row r="14" spans="1:4" ht="18" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="7"/>
-    </row>
-    <row r="15" spans="1:4" ht="18" customHeight="1">
-      <c r="A15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="7"/>
-    </row>
-    <row r="16" spans="1:4" ht="20.399999999999999">
-      <c r="A16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="7"/>
-    </row>
-    <row r="17" spans="1:4" ht="18" customHeight="1">
-      <c r="A17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="7"/>
-    </row>
-    <row r="18" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="7"/>
-    </row>
-    <row r="19" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A19" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="7"/>
-    </row>
-    <row r="20" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="7"/>
-    </row>
-    <row r="21" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="7"/>
-    </row>
-    <row r="22" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="7"/>
-    </row>
-    <row r="23" spans="1:4" ht="18" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" ht="18" customHeight="1">
-      <c r="A24" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="7"/>
-    </row>
-    <row r="25" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="7"/>
-    </row>
-    <row r="26" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A26" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="7"/>
-    </row>
-    <row r="27" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A27" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="7"/>
-    </row>
-    <row r="28" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A28" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="7"/>
-    </row>
-    <row r="29" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="7"/>
-    </row>
-    <row r="30" spans="1:4" ht="18" customHeight="1">
-      <c r="A30" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="25"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="7"/>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A31" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="7"/>
-    </row>
-    <row r="32" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A32" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="7"/>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A33" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="25"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="7"/>
-    </row>
-    <row r="34" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A34" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B34" s="25"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="7"/>
-    </row>
-    <row r="35" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A35" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B35" s="25"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="7"/>
-    </row>
-    <row r="36" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A36" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="7"/>
-    </row>
-    <row r="37" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A37" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B37" s="25"/>
+      <c r="B37" s="27" t="s">
+        <v>15</v>
+      </c>
       <c r="C37" s="26"/>
-      <c r="D37" s="7"/>
-    </row>
-    <row r="38" spans="1:4" ht="18" customHeight="1">
+      <c r="D37" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="30" customHeight="1">
       <c r="A38" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="25"/>
+        <v>40</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>15</v>
+      </c>
       <c r="C38" s="26"/>
-      <c r="D38" s="7"/>
-    </row>
-    <row r="39" spans="1:4" ht="20.25" customHeight="1">
+      <c r="D38" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="30" customHeight="1">
       <c r="A39" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="27"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="7"/>
-    </row>
-    <row r="40" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A40" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="7"/>
-    </row>
-    <row r="41" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A41" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B41" s="25"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="7"/>
-    </row>
-    <row r="42" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A42" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B42" s="25"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="7"/>
-    </row>
-    <row r="43" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A43" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B43" s="25"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="7"/>
+      <c r="B39" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="26"/>
+      <c r="D39" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="30" customHeight="1">
+      <c r="A40" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="26"/>
+      <c r="D40" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="30" customHeight="1">
+      <c r="A41" s="9"/>
+      <c r="B41" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" s="11">
+        <v>0</v>
+      </c>
+      <c r="D41" s="12"/>
+    </row>
+    <row r="42" spans="1:4" ht="30" customHeight="1">
+      <c r="A42" s="9"/>
+      <c r="B42" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" s="11">
+        <v>0</v>
+      </c>
+      <c r="D42" s="12"/>
+    </row>
+    <row r="43" spans="1:4" ht="15" customHeight="1">
+      <c r="B43" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="44" spans="1:4" ht="15" customHeight="1">
-      <c r="B44" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>35</v>
-      </c>
+      <c r="B44" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="15"/>
     </row>
     <row r="45" spans="1:4" ht="15" customHeight="1">
-      <c r="B45" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C45" s="13" t="s">
-        <v>36</v>
+      <c r="B45" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15" customHeight="1">
-      <c r="B46" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15" customHeight="1">
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
-    </row>
-    <row r="48" spans="1:4" ht="15.75" customHeight="1">
-      <c r="B48" s="32"/>
-      <c r="C48" s="32"/>
-    </row>
-    <row r="49" spans="2:3" ht="15.75" customHeight="1">
-      <c r="B49" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C49" s="15" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="50" spans="2:3" ht="15.75" customHeight="1">
-      <c r="B50" s="33"/>
+      <c r="B46" s="32"/>
+      <c r="C46" s="32"/>
+    </row>
+    <row r="47" spans="1:4" ht="14.25" customHeight="1">
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+    </row>
+    <row r="48" spans="1:4" ht="14.25" customHeight="1">
+      <c r="B48" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B49" s="36"/>
+      <c r="C49" s="34"/>
+    </row>
+    <row r="50" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B50" s="35"/>
       <c r="C50" s="35"/>
     </row>
-    <row r="51" spans="2:3" ht="15.75" customHeight="1">
-      <c r="B51" s="34"/>
-      <c r="C51" s="34"/>
-    </row>
-    <row r="52" spans="2:3" ht="15.75" customHeight="1">
-      <c r="B52" s="32"/>
-      <c r="C52" s="32"/>
-    </row>
-    <row r="53" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="54" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="55" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="56" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="57" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="58" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="59" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="60" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="61" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="62" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="63" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="64" spans="2:3" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="51" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B51" s="35"/>
+      <c r="C51" s="35"/>
+    </row>
+    <row r="52" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+    </row>
+    <row r="53" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
+    </row>
+    <row r="54" spans="2:3" ht="14.25" customHeight="1">
+      <c r="B54" s="33"/>
+      <c r="C54" s="33"/>
+    </row>
+    <row r="55" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="56" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="57" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="58" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="59" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="60" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="62" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="63" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="64" spans="2:3" ht="14.25" customHeight="1"/>
+    <row r="65" ht="14.25" customHeight="1"/>
+    <row r="66" ht="14.25" customHeight="1"/>
+    <row r="67" ht="14.25" customHeight="1"/>
+    <row r="68" ht="14.25" customHeight="1"/>
+    <row r="69" ht="14.25" customHeight="1"/>
+    <row r="70" ht="14.25" customHeight="1"/>
+    <row r="71" ht="14.25" customHeight="1"/>
+    <row r="72" ht="14.25" customHeight="1"/>
+    <row r="73" ht="14.25" customHeight="1"/>
+    <row r="74" ht="14.25" customHeight="1"/>
+    <row r="75" ht="14.25" customHeight="1"/>
+    <row r="76" ht="14.25" customHeight="1"/>
+    <row r="77" ht="14.25" customHeight="1"/>
+    <row r="78" ht="14.25" customHeight="1"/>
+    <row r="79" ht="14.25" customHeight="1"/>
+    <row r="80" ht="14.25" customHeight="1"/>
+    <row r="81" ht="14.25" customHeight="1"/>
+    <row r="82" ht="14.25" customHeight="1"/>
+    <row r="83" ht="14.25" customHeight="1"/>
+    <row r="84" ht="14.25" customHeight="1"/>
+    <row r="85" ht="14.25" customHeight="1"/>
+    <row r="86" ht="14.25" customHeight="1"/>
+    <row r="87" ht="14.25" customHeight="1"/>
+    <row r="88" ht="14.25" customHeight="1"/>
+    <row r="89" ht="14.25" customHeight="1"/>
+    <row r="90" ht="14.25" customHeight="1"/>
+    <row r="91" ht="14.25" customHeight="1"/>
+    <row r="92" ht="14.25" customHeight="1"/>
+    <row r="93" ht="14.25" customHeight="1"/>
+    <row r="94" ht="14.25" customHeight="1"/>
+    <row r="95" ht="14.25" customHeight="1"/>
+    <row r="96" ht="14.25" customHeight="1"/>
+    <row r="97" ht="14.25" customHeight="1"/>
+    <row r="98" ht="14.25" customHeight="1"/>
+    <row r="99" ht="14.25" customHeight="1"/>
+    <row r="100" ht="14.25" customHeight="1"/>
+    <row r="101" ht="14.25" customHeight="1"/>
+    <row r="102" ht="14.25" customHeight="1"/>
+    <row r="103" ht="14.25" customHeight="1"/>
+    <row r="104" ht="14.25" customHeight="1"/>
+    <row r="105" ht="14.25" customHeight="1"/>
+    <row r="106" ht="14.25" customHeight="1"/>
+    <row r="107" ht="14.25" customHeight="1"/>
+    <row r="108" ht="14.25" customHeight="1"/>
+    <row r="109" ht="14.25" customHeight="1"/>
+    <row r="110" ht="14.25" customHeight="1"/>
+    <row r="111" ht="14.25" customHeight="1"/>
+    <row r="112" ht="14.25" customHeight="1"/>
+    <row r="113" ht="14.25" customHeight="1"/>
+    <row r="114" ht="14.25" customHeight="1"/>
+    <row r="115" ht="14.25" customHeight="1"/>
+    <row r="116" ht="14.25" customHeight="1"/>
+    <row r="117" ht="14.25" customHeight="1"/>
+    <row r="118" ht="14.25" customHeight="1"/>
+    <row r="119" ht="14.25" customHeight="1"/>
+    <row r="120" ht="14.25" customHeight="1"/>
+    <row r="121" ht="14.25" customHeight="1"/>
+    <row r="122" ht="14.25" customHeight="1"/>
+    <row r="123" ht="14.25" customHeight="1"/>
+    <row r="124" ht="14.25" customHeight="1"/>
+    <row r="125" ht="14.25" customHeight="1"/>
+    <row r="126" ht="14.25" customHeight="1"/>
+    <row r="127" ht="14.25" customHeight="1"/>
+    <row r="128" ht="14.25" customHeight="1"/>
+    <row r="129" ht="14.25" customHeight="1"/>
+    <row r="130" ht="14.25" customHeight="1"/>
+    <row r="131" ht="14.25" customHeight="1"/>
+    <row r="132" ht="14.25" customHeight="1"/>
+    <row r="133" ht="14.25" customHeight="1"/>
+    <row r="134" ht="14.25" customHeight="1"/>
+    <row r="135" ht="14.25" customHeight="1"/>
+    <row r="136" ht="14.25" customHeight="1"/>
+    <row r="137" ht="14.25" customHeight="1"/>
+    <row r="138" ht="14.25" customHeight="1"/>
+    <row r="139" ht="14.25" customHeight="1"/>
+    <row r="140" ht="14.25" customHeight="1"/>
+    <row r="141" ht="14.25" customHeight="1"/>
+    <row r="142" ht="14.25" customHeight="1"/>
+    <row r="143" ht="14.25" customHeight="1"/>
+    <row r="144" ht="14.25" customHeight="1"/>
+    <row r="145" ht="14.25" customHeight="1"/>
+    <row r="146" ht="14.25" customHeight="1"/>
+    <row r="147" ht="14.25" customHeight="1"/>
+    <row r="148" ht="14.25" customHeight="1"/>
+    <row r="149" ht="14.25" customHeight="1"/>
+    <row r="150" ht="14.25" customHeight="1"/>
+    <row r="151" ht="14.25" customHeight="1"/>
+    <row r="152" ht="14.25" customHeight="1"/>
+    <row r="153" ht="14.25" customHeight="1"/>
+    <row r="154" ht="14.25" customHeight="1"/>
+    <row r="155" ht="14.25" customHeight="1"/>
+    <row r="156" ht="14.25" customHeight="1"/>
+    <row r="157" ht="14.25" customHeight="1"/>
+    <row r="158" ht="14.25" customHeight="1"/>
+    <row r="159" ht="14.25" customHeight="1"/>
+    <row r="160" ht="14.25" customHeight="1"/>
+    <row r="161" ht="14.25" customHeight="1"/>
+    <row r="162" ht="14.25" customHeight="1"/>
+    <row r="163" ht="14.25" customHeight="1"/>
+    <row r="164" ht="14.25" customHeight="1"/>
+    <row r="165" ht="14.25" customHeight="1"/>
+    <row r="166" ht="14.25" customHeight="1"/>
+    <row r="167" ht="14.25" customHeight="1"/>
+    <row r="168" ht="14.25" customHeight="1"/>
+    <row r="169" ht="14.25" customHeight="1"/>
+    <row r="170" ht="14.25" customHeight="1"/>
+    <row r="171" ht="14.25" customHeight="1"/>
+    <row r="172" ht="14.25" customHeight="1"/>
+    <row r="173" ht="14.25" customHeight="1"/>
+    <row r="174" ht="14.25" customHeight="1"/>
+    <row r="175" ht="14.25" customHeight="1"/>
+    <row r="176" ht="14.25" customHeight="1"/>
+    <row r="177" ht="14.25" customHeight="1"/>
+    <row r="178" ht="14.25" customHeight="1"/>
+    <row r="179" ht="14.25" customHeight="1"/>
+    <row r="180" ht="14.25" customHeight="1"/>
+    <row r="181" ht="14.25" customHeight="1"/>
+    <row r="182" ht="14.25" customHeight="1"/>
+    <row r="183" ht="14.25" customHeight="1"/>
+    <row r="184" ht="14.25" customHeight="1"/>
+    <row r="185" ht="14.25" customHeight="1"/>
+    <row r="186" ht="14.25" customHeight="1"/>
+    <row r="187" ht="14.25" customHeight="1"/>
+    <row r="188" ht="14.25" customHeight="1"/>
+    <row r="189" ht="14.25" customHeight="1"/>
+    <row r="190" ht="14.25" customHeight="1"/>
+    <row r="191" ht="14.25" customHeight="1"/>
+    <row r="192" ht="14.25" customHeight="1"/>
+    <row r="193" ht="14.25" customHeight="1"/>
+    <row r="194" ht="14.25" customHeight="1"/>
+    <row r="195" ht="14.25" customHeight="1"/>
+    <row r="196" ht="14.25" customHeight="1"/>
+    <row r="197" ht="14.25" customHeight="1"/>
+    <row r="198" ht="14.25" customHeight="1"/>
+    <row r="199" ht="14.25" customHeight="1"/>
+    <row r="200" ht="14.25" customHeight="1"/>
+    <row r="201" ht="14.25" customHeight="1"/>
+    <row r="202" ht="14.25" customHeight="1"/>
+    <row r="203" ht="14.25" customHeight="1"/>
+    <row r="204" ht="14.25" customHeight="1"/>
+    <row r="205" ht="14.25" customHeight="1"/>
+    <row r="206" ht="14.25" customHeight="1"/>
+    <row r="207" ht="14.25" customHeight="1"/>
+    <row r="208" ht="14.25" customHeight="1"/>
+    <row r="209" ht="14.25" customHeight="1"/>
+    <row r="210" ht="14.25" customHeight="1"/>
+    <row r="211" ht="14.25" customHeight="1"/>
+    <row r="212" ht="14.25" customHeight="1"/>
+    <row r="213" ht="14.25" customHeight="1"/>
+    <row r="214" ht="14.25" customHeight="1"/>
+    <row r="215" ht="14.25" customHeight="1"/>
+    <row r="216" ht="14.25" customHeight="1"/>
+    <row r="217" ht="14.25" customHeight="1"/>
+    <row r="218" ht="14.25" customHeight="1"/>
+    <row r="219" ht="14.25" customHeight="1"/>
+    <row r="220" ht="14.25" customHeight="1"/>
+    <row r="221" ht="14.25" customHeight="1"/>
+    <row r="222" ht="14.25" customHeight="1"/>
+    <row r="223" ht="14.25" customHeight="1"/>
+    <row r="224" ht="14.25" customHeight="1"/>
+    <row r="225" ht="14.25" customHeight="1"/>
+    <row r="226" ht="14.25" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
+    <row r="228" ht="14.25" customHeight="1"/>
+    <row r="229" ht="14.25" customHeight="1"/>
+    <row r="230" ht="14.25" customHeight="1"/>
+    <row r="231" ht="14.25" customHeight="1"/>
+    <row r="232" ht="14.25" customHeight="1"/>
+    <row r="233" ht="14.25" customHeight="1"/>
+    <row r="234" ht="14.25" customHeight="1"/>
+    <row r="235" ht="14.25" customHeight="1"/>
+    <row r="236" ht="14.25" customHeight="1"/>
+    <row r="237" ht="14.25" customHeight="1"/>
+    <row r="238" ht="14.25" customHeight="1"/>
+    <row r="239" ht="14.25" customHeight="1"/>
+    <row r="240" ht="14.25" customHeight="1"/>
+    <row r="241" ht="14.25" customHeight="1"/>
+    <row r="242" ht="14.25" customHeight="1"/>
+    <row r="243" ht="14.25" customHeight="1"/>
+    <row r="244" ht="14.25" customHeight="1"/>
+    <row r="245" ht="14.25" customHeight="1"/>
+    <row r="246" ht="14.25" customHeight="1"/>
+    <row r="247" ht="14.25" customHeight="1"/>
+    <row r="248" ht="14.25" customHeight="1"/>
     <row r="249" ht="15.75" customHeight="1"/>
     <row r="250" ht="15.75" customHeight="1"/>
     <row r="251" ht="15.75" customHeight="1"/>
@@ -2209,21 +2365,10 @@
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="B50:B52"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
+  <mergeCells count="39">
+    <mergeCell ref="C49:C54"/>
+    <mergeCell ref="B49:B54"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
@@ -2231,6 +2376,11 @@
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
@@ -2263,5 +2413,6 @@
     <oddHeader>&amp;L06-049DIRECTION SYSTEME D'INFORMATION</oddHeader>
     <oddFooter>&amp;RPage &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>